<commit_message>
Remove a exigência de vice-líder de outro período nas equipes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MBn9YrntdXfTASAVKo9hpN
</commit_message>
<xml_diff>
--- a/entregas/equipes/planilha-equipes.xlsx
+++ b/entregas/equipes/planilha-equipes.xlsx
@@ -771,7 +771,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Vice-líder (outro período)</t>
+          <t>Vice-líder</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Vice-líder (outro período)</t>
+          <t>Vice-líder</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Vice-líder (outro período)</t>
+          <t>Vice-líder</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Vice-líder (outro período)</t>
+          <t>Vice-líder</t>
         </is>
       </c>
       <c r="C58" t="n">

</xml_diff>

<commit_message>
Mensagens de WhatsApp no padrão da turma, líderes definidos e vice no Financeiro
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MBn9YrntdXfTASAVKo9hpN
</commit_message>
<xml_diff>
--- a/entregas/equipes/planilha-equipes.xlsx
+++ b/entregas/equipes/planilha-equipes.xlsx
@@ -1635,7 +1635,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Conferência de repasses</t>
+          <t>Vice-líder</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr"/>
@@ -1671,11 +1671,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Compras e notas fiscais</t>
+          <t>Conferência de repasses</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr"/>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Despesas e comprovantes</t>
+          <t>Compras e notas fiscais</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Transparência</t>
+          <t>Despesas e comprovantes</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -1718,40 +1718,40 @@
       <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>Triagem e Aferição dos Itens</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Financeiro e Prestação de Contas</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Transparência</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Triagem e Aferição dos Itens</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
         <is>
           <t>Líder</t>
         </is>
       </c>
-      <c r="C57" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D57" s="4" t="inlineStr"/>
-      <c r="E57" s="4" t="inlineStr"/>
-      <c r="F57" s="4" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Triagem e Aferição dos Itens</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Vice-líder</t>
-        </is>
-      </c>
-      <c r="C58" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
+      <c r="C58" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="4" t="inlineStr"/>
+      <c r="E58" s="4" t="inlineStr"/>
+      <c r="F58" s="4" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Recolhimento no campus</t>
+          <t>Vice-líder</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -1783,7 +1783,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr"/>
@@ -1801,7 +1801,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr"/>
@@ -1819,7 +1819,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
@@ -1833,11 +1833,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Recolhimento nos parceiros</t>
+          <t>Recolhimento no campus</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr"/>
@@ -1855,7 +1855,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr"/>
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr"/>
@@ -1891,7 +1891,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr"/>
@@ -1909,7 +1909,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr"/>
@@ -1923,11 +1923,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Triagem e conformidade</t>
+          <t>Recolhimento nos parceiros</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr"/>
@@ -1945,7 +1945,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr"/>
@@ -1963,7 +1963,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr"/>
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr"/>
@@ -1999,7 +1999,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr"/>
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr"/>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr"/>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr"/>

</xml_diff>